<commit_message>
Velocidad vertical por helicóptero en el modelo de tiempo y costo
- Nuevo campo vertical_speed_ms: cada despegue+aterrizaje suma el tiempo de
  ascenso y descenso a la altitud de crucero (cruise_altitude_m, 300 m por
  defecto, configurable en Config del Excel y en JSON).
- Horas de tramo = km/velocidad crucero + 2×altitud/velocidad vertical: el
  perfil de pedidos decide el modelo (tramos largos → crucero rápido; muchas
  paradas → ascenso rápido y hora barata).
- Catálogo con regímenes de ascenso típicos (Mi-171 8.0, Bell 412 6.9,
  H145 8.1, BK117 8.4, H125 9.0 m/s); columna nueva en la hoja Helicopteros.
- El salto de seguridad de combustible también incluye el tiempo vertical.
- 2 tests nuevos (37 en total), incluido uno donde el helicóptero de ascenso
  rápido gana pese a tarifa mayor.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011nqEw3XJGAAL7PxhmbC5nJ
</commit_message>
<xml_diff>
--- a/examples/entrada_malvinas.xlsx
+++ b/examples/entrada_malvinas.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,22 +458,32 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Regreso a base</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
+          <t>Altitud de crucero (m)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
+          <t>Regreso a base</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
           <t>Hora inicio</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
@@ -1020,7 +1030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1087,6 +1097,11 @@
       <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Tamaño (1-3)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Vel. vertical (m/s)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tiempo en tierra admisible por helicóptero y estadísticas por cliente
- Nuevo campo free_ground_min por helicóptero: minutos de escala incluidos
  en la tarifa; el exceso se factura al cliente de la parada a la tarifa
  horaria y se reporta como cargo separado.
- Estimación del tiempo en tierra por parada: base + min/pax + min/100 kg
  (configurable en Config); corre el horario de la programación.
- plan_visits y ground_stats_by_company en el optimizador: por empresa se
  obtiene paradas, tiempo en tierra mín/promedio/máx, exceso y cargo total.
- Excel: hoja nueva 'Tiempo en tierra' (detalle por parada + resumen por
  empresa), línea 'En tierra X min' por parada en la Programación, columna
  'T. tierra admisible (min)' en Helicopteros.
- CLI: resumen de tiempo en tierra por cliente tras el plan óptimo.
- 2 tests nuevos (39 en total).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011nqEw3XJGAAL7PxhmbC5nJ
</commit_message>
<xml_diff>
--- a/examples/entrada_malvinas.xlsx
+++ b/examples/entrada_malvinas.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,22 +468,52 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Regreso a base</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
+          <t>Minutos base por parada</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
+          <t>Minutos por pax</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Minutos por 100 kg</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Regreso a base</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
           <t>Hora inicio</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
@@ -1030,7 +1060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1104,6 +1134,11 @@
           <t>Vel. vertical (m/s)</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>T. tierra admisible (min)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1132,6 +1167,9 @@
           <t>SI</t>
         </is>
       </c>
+      <c r="O2" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1157,6 +1195,9 @@
           <t>SI</t>
         </is>
       </c>
+      <c r="O3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1181,6 +1222,9 @@
         <is>
           <t>SI</t>
         </is>
+      </c>
+      <c r="O4" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>